<commit_message>
Enforce unique inventory numbers
</commit_message>
<xml_diff>
--- a/workbook/Lutherska-Inventarier.xlsx
+++ b/workbook/Lutherska-Inventarier.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
   <si>
     <t>Id</t>
   </si>
@@ -26,6 +26,9 @@
     <t>Color</t>
   </si>
   <si>
+    <t>Prefix</t>
+  </si>
+  <si>
     <t>cat-furniture</t>
   </si>
   <si>
@@ -35,6 +38,9 @@
     <t>#6f8657</t>
   </si>
   <si>
+    <t>MOB</t>
+  </si>
+  <si>
     <t>cat-lighting</t>
   </si>
   <si>
@@ -44,6 +50,9 @@
     <t>#f59b45</t>
   </si>
   <si>
+    <t>BEL</t>
+  </si>
+  <si>
     <t>cat-sound</t>
   </si>
   <si>
@@ -53,6 +62,9 @@
     <t>#3688df</t>
   </si>
   <si>
+    <t>LJU</t>
+  </si>
+  <si>
     <t>cat-kitchen</t>
   </si>
   <si>
@@ -60,6 +72,9 @@
   </si>
   <si>
     <t>#c73f3b</t>
+  </si>
+  <si>
+    <t>KOK</t>
   </si>
   <si>
     <t>grp-board-mission</t>
@@ -330,16 +345,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Categories" displayName="Categories" ref="A1:C5" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:C5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Categories" displayName="Categories" ref="A1:D5" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:D5">
     <filterColumn colId="0" hiddenButton="0"/>
     <filterColumn colId="1" hiddenButton="0"/>
     <filterColumn colId="2" hiddenButton="0"/>
+    <filterColumn colId="3" hiddenButton="0"/>
   </autoFilter>
-  <tableColumns count="3">
+  <tableColumns count="4">
     <tableColumn id="1" name="Id" totalsRowLabel="Total"/>
     <tableColumn id="2" name="Name" totalsRowFunction="none"/>
     <tableColumn id="3" name="Color" totalsRowFunction="none"/>
+    <tableColumn id="4" name="Prefix" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -749,15 +766,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="19" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -767,49 +785,64 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -840,186 +873,186 @@
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1050,34 +1083,34 @@
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1110,31 +1143,36 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="error" errorTitle="Ogiltigt inventarienummer" error="Använd kategorins trebokstavskod, bindestreck och tre siffror. Numret måste vara unikt, till exempel MOB-014." sqref="B2:B5000">
+      <formula1>=OR(COUNTA(A2:I2)=0,AND(LEN(B2)=7,MID(B2,4,1)="-",CODE(MID(B2,1,1))&gt;=65,CODE(MID(B2,1,1))&lt;=90,CODE(MID(B2,2,1))&gt;=65,CODE(MID(B2,2,1))&lt;=90,CODE(MID(B2,3,1))&gt;=65,CODE(MID(B2,3,1))&lt;=90,ISNUMBER(--RIGHT(B2,3)),COUNTIF($B:$B,B2)=1,D2&lt;&gt;"",LEFT(B2,3)=IFERROR(VLOOKUP(D2,Categories,4,FALSE),"")))</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
@@ -1160,25 +1198,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>